<commit_message>
chore(oscal): add basic-catalog.yaml test
</commit_message>
<xml_diff>
--- a/project/excel/nist_sp_800_53.xlsx
+++ b/project/excel/nist_sp_800_53.xlsx
@@ -693,74 +693,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>controls</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>_class</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>props</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>links</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>parts</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"family,SP800-53,SP800-53-enhancement"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>params</t>
+          <t>groups</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -814,7 +753,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -880,28 +819,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>catalog</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -913,12 +831,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>guidelines</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>select</t>
+          <t>params</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>controls</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -967,6 +885,93 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>catalog</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>guidelines</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>select</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>_class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>props</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>links</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>parts</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"family,SP800-53,SP800-53-enhancement"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(nist): add cprt support in schema and tests
</commit_message>
<xml_diff>
--- a/project/excel/nist_sp_800_53.xlsx
+++ b/project/excel/nist_sp_800_53.xlsx
@@ -35,6 +35,15 @@
     <sheet name="ImportResource" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="IncludeControlsSelection" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="MergeRules" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="FlatMerge" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="ControlPattern" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="ExcludeControlsSelection" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="ProfileModify" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="ProfileSetParameter" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="ProfileAlter" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="ProfileAdd" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="CPRTDocument" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="CPRTResponse" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -440,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +461,11 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>profile</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>response</t>
         </is>
       </c>
     </row>
@@ -680,7 +694,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"family,SP800-53,SP800-53-enhancement"</formula1>
+      <formula1>"family,SP800-53,SP800-53-enhancement,assessment-objective"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -746,7 +760,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"family,SP800-53,SP800-53-enhancement"</formula1>
+      <formula1>"family,SP800-53,SP800-53-enhancement,assessment-objective"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -812,7 +826,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"family,SP800-53,SP800-53-enhancement"</formula1>
+      <formula1>"family,SP800-53,SP800-53-enhancement,assessment-objective"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -878,7 +892,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"family,SP800-53,SP800-53-enhancement"</formula1>
+      <formula1>"family,SP800-53,SP800-53-enhancement,assessment-objective"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -912,7 +926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -928,35 +942,40 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>depends-on</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>_class</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>props</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>links</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>parts</t>
         </is>
@@ -964,8 +983,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"family,SP800-53,SP800-53-enhancement"</formula1>
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"family,SP800-53,SP800-53-enhancement,assessment-objective"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1145,7 +1164,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"family,SP800-53,SP800-53-enhancement"</formula1>
+      <formula1>"family,SP800-53,SP800-53-enhancement,assessment-objective"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1158,27 +1177,84 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>href</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>include-controls</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>exclude-controls</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>href</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>include-controls</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>with-ids</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>matching</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>as-is</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1186,6 +1262,61 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1193,13 +1324,132 @@
           <t>with-ids</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>matching</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>set-parameters</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>alters</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>param-id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>control-id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>adds</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>by-id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>parts</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>props</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1211,16 +1461,16 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>as-is</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>response</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1228,15 +1478,7 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>profile</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1283,7 +1525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1309,6 +1551,11 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>modify</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>back-matter</t>
         </is>
       </c>

</xml_diff>